<commit_message>
chore: sync workbook from OneDrive
</commit_message>
<xml_diff>
--- a/data/report.xlsx
+++ b/data/report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bank Muscat\AD Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="390" documentId="13_ncr:1_{4A272BF1-49BC-4E00-83C3-F2030B573C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95D7CB3C-75A2-40C6-B5DD-5CECF53324A3}"/>
+  <xr:revisionPtr revIDLastSave="395" documentId="13_ncr:1_{4A272BF1-49BC-4E00-83C3-F2030B573C9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89024CE3-EC2F-4ED2-82FB-9464D4955AF4}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="278">
   <si>
     <t>Client / entity</t>
   </si>
@@ -909,6 +909,12 @@
   </si>
   <si>
     <t>LLMApp /getResponse JSON consumed by the AD SOE portal; DataApp Postgres tables per measure + analysis cache; IOApp markdown of uploaded documents in MinIO; MinIOApp document list/get/delete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Test </t>
+  </si>
+  <si>
+    <t>Anomaly Deyection in Bank</t>
   </si>
 </sst>
 </file>
@@ -1050,7 +1056,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1138,12 +1144,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1217,9 +1247,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1244,9 +1271,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1264,6 +1288,36 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1589,7 +1643,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AG12"/>
+  <dimension ref="A1:AG13"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="18.7109375" style="23" customWidth="1"/>
@@ -1714,21 +1768,21 @@
       <c r="AB1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="31" t="s">
+      <c r="AC1" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="27" t="s">
+      <c r="AD1" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="27" t="s">
+      <c r="AE1" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="27" t="s">
+      <c r="AF1" s="26" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:33" s="14" customFormat="1" ht="166.5">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="33" t="s">
         <v>32</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1810,17 +1864,17 @@
       <c r="AB2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="AC2" s="32" t="s">
+      <c r="AC2" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="AD2" s="28"/>
-      <c r="AE2" s="28"/>
-      <c r="AF2" s="28" t="s">
+      <c r="AD2" s="27"/>
+      <c r="AE2" s="27"/>
+      <c r="AF2" s="27" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:33" s="14" customFormat="1" ht="130.5">
-      <c r="A3" s="36"/>
+      <c r="A3" s="34"/>
       <c r="B3" s="1" t="s">
         <v>61</v>
       </c>
@@ -1900,12 +1954,12 @@
       <c r="AB3" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="AC3" s="32" t="s">
+      <c r="AC3" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="AD3" s="28"/>
-      <c r="AE3" s="28"/>
-      <c r="AF3" s="28" t="s">
+      <c r="AD3" s="27"/>
+      <c r="AE3" s="27"/>
+      <c r="AF3" s="27" t="s">
         <v>60</v>
       </c>
       <c r="AG3" s="14" t="s">
@@ -1913,7 +1967,7 @@
       </c>
     </row>
     <row r="4" spans="1:33" s="17" customFormat="1" ht="63.6" customHeight="1">
-      <c r="A4" s="37"/>
+      <c r="A4" s="35"/>
       <c r="B4" s="1" t="s">
         <v>72</v>
       </c>
@@ -1985,12 +2039,12 @@
       <c r="AB4" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="AC4" s="33" t="s">
+      <c r="AC4" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="AD4" s="29"/>
-      <c r="AE4" s="29"/>
-      <c r="AF4" s="28" t="s">
+      <c r="AD4" s="28"/>
+      <c r="AE4" s="28"/>
+      <c r="AF4" s="27" t="s">
         <v>60</v>
       </c>
       <c r="AG4" s="14" t="s">
@@ -1998,7 +2052,7 @@
       </c>
     </row>
     <row r="5" spans="1:33" s="17" customFormat="1" ht="84">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="36" t="s">
         <v>89</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -2082,15 +2136,15 @@
       <c r="AB5" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="AC5" s="33" t="s">
+      <c r="AC5" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="AD5" s="29"/>
-      <c r="AE5" s="29"/>
-      <c r="AF5" s="29"/>
+      <c r="AD5" s="28"/>
+      <c r="AE5" s="28"/>
+      <c r="AF5" s="28"/>
     </row>
     <row r="6" spans="1:33" s="17" customFormat="1" ht="84">
-      <c r="A6" s="39"/>
+      <c r="A6" s="37"/>
       <c r="B6" s="15" t="s">
         <v>117</v>
       </c>
@@ -2172,15 +2226,15 @@
       <c r="AB6" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="AC6" s="33" t="s">
+      <c r="AC6" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="AD6" s="29"/>
-      <c r="AE6" s="29"/>
-      <c r="AF6" s="29"/>
+      <c r="AD6" s="28"/>
+      <c r="AE6" s="28"/>
+      <c r="AF6" s="28"/>
     </row>
     <row r="7" spans="1:33" s="17" customFormat="1" ht="72">
-      <c r="A7" s="40"/>
+      <c r="A7" s="38"/>
       <c r="B7" s="15" t="s">
         <v>142</v>
       </c>
@@ -2262,15 +2316,15 @@
       <c r="AB7" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="AC7" s="33" t="s">
+      <c r="AC7" s="32" t="s">
         <v>166</v>
       </c>
-      <c r="AD7" s="29"/>
-      <c r="AE7" s="29"/>
-      <c r="AF7" s="29"/>
+      <c r="AD7" s="28"/>
+      <c r="AE7" s="28"/>
+      <c r="AF7" s="28"/>
     </row>
     <row r="8" spans="1:33" ht="130.5" customHeight="1">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="36" t="s">
         <v>167</v>
       </c>
       <c r="B8" s="15" t="s">
@@ -2354,18 +2408,18 @@
       <c r="AB8" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="AC8" s="33" t="s">
+      <c r="AC8" s="32" t="s">
         <v>194</v>
       </c>
-      <c r="AD8" s="29"/>
-      <c r="AE8" s="29"/>
-      <c r="AF8" s="28" t="s">
+      <c r="AD8" s="28"/>
+      <c r="AE8" s="28"/>
+      <c r="AF8" s="27" t="s">
         <v>195</v>
       </c>
       <c r="AG8" s="17"/>
     </row>
     <row r="9" spans="1:33" s="23" customFormat="1" ht="122.25" customHeight="1">
-      <c r="A9" s="40"/>
+      <c r="A9" s="38"/>
       <c r="B9" s="15" t="s">
         <v>196</v>
       </c>
@@ -2375,7 +2429,7 @@
       <c r="D9" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="25" t="s">
         <v>198</v>
       </c>
       <c r="F9" s="16" t="s">
@@ -2433,12 +2487,12 @@
         <v>214</v>
       </c>
       <c r="AB9" s="16"/>
-      <c r="AC9" s="33" t="s">
+      <c r="AC9" s="32" t="s">
         <v>215</v>
       </c>
-      <c r="AD9" s="30"/>
-      <c r="AE9" s="30"/>
-      <c r="AF9" s="28" t="s">
+      <c r="AD9" s="29"/>
+      <c r="AE9" s="29"/>
+      <c r="AF9" s="27" t="s">
         <v>216</v>
       </c>
     </row>
@@ -2527,14 +2581,14 @@
       <c r="AB10" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="AC10" s="33" t="s">
+      <c r="AC10" s="32" t="s">
         <v>224</v>
       </c>
-      <c r="AD10" s="29"/>
-      <c r="AE10" s="29" t="s">
+      <c r="AD10" s="28"/>
+      <c r="AE10" s="28" t="s">
         <v>232</v>
       </c>
-      <c r="AF10" s="29" t="s">
+      <c r="AF10" s="28" t="s">
         <v>233</v>
       </c>
     </row>
@@ -2623,105 +2677,147 @@
       <c r="AB11" s="15" t="s">
         <v>260</v>
       </c>
-      <c r="AC11" s="33"/>
-      <c r="AD11" s="29"/>
-      <c r="AE11" s="29"/>
-      <c r="AF11" s="29"/>
+      <c r="AC11" s="32"/>
+      <c r="AD11" s="28"/>
+      <c r="AE11" s="28"/>
+      <c r="AF11" s="28"/>
       <c r="AG11" s="17"/>
     </row>
     <row r="12" spans="1:33" s="17" customFormat="1" ht="195" customHeight="1">
-      <c r="A12" s="25" t="s">
+      <c r="A12" s="41" t="s">
         <v>261</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="42" t="s">
         <v>262</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="42" t="s">
         <v>263</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="42" t="s">
         <v>264</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="42" t="s">
         <v>266</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="G12" s="42" t="s">
         <v>267</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="H12" s="42" t="s">
         <v>268</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="42" t="s">
         <v>224</v>
       </c>
-      <c r="J12" s="18" t="s">
+      <c r="J12" s="44" t="s">
         <v>224</v>
       </c>
-      <c r="K12" s="16" t="s">
+      <c r="K12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="L12" s="16" t="s">
+      <c r="L12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="M12" s="16" t="s">
+      <c r="M12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="N12" s="16" t="s">
+      <c r="N12" s="45" t="s">
         <v>269</v>
       </c>
-      <c r="O12" s="16" t="s">
+      <c r="O12" s="45" t="s">
         <v>270</v>
       </c>
-      <c r="P12" s="15" t="s">
+      <c r="P12" s="42" t="s">
         <v>271</v>
       </c>
-      <c r="Q12" s="16" t="s">
+      <c r="Q12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="R12" s="16" t="s">
+      <c r="R12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="S12" s="16" t="s">
+      <c r="S12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="T12" s="15" t="s">
+      <c r="T12" s="42" t="s">
         <v>272</v>
       </c>
-      <c r="U12" s="16" t="s">
+      <c r="U12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="V12" s="16" t="s">
+      <c r="V12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="W12" s="16" t="s">
+      <c r="W12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="X12" s="16" t="s">
+      <c r="X12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="Y12" s="15" t="s">
+      <c r="Y12" s="42" t="s">
         <v>273</v>
       </c>
-      <c r="Z12" s="15" t="s">
+      <c r="Z12" s="42" t="s">
         <v>274</v>
       </c>
-      <c r="AA12" s="15" t="s">
+      <c r="AA12" s="42" t="s">
         <v>275</v>
       </c>
-      <c r="AB12" s="16" t="s">
+      <c r="AB12" s="45" t="s">
         <v>224</v>
       </c>
-      <c r="AC12" s="34" t="s">
+      <c r="AC12" s="46" t="s">
         <v>224</v>
       </c>
-      <c r="AD12" s="29"/>
-      <c r="AE12" s="29"/>
-      <c r="AF12" s="28" t="s">
+      <c r="AD12" s="47"/>
+      <c r="AE12" s="47"/>
+      <c r="AF12" s="48" t="s">
         <v>216</v>
       </c>
+    </row>
+    <row r="13" spans="1:33" ht="24">
+      <c r="A13" s="29" t="s">
+        <v>276</v>
+      </c>
+      <c r="B13" s="39" t="s">
+        <v>277</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="40"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
+      <c r="N13" s="40"/>
+      <c r="O13" s="39"/>
+      <c r="P13" s="39"/>
+      <c r="Q13" s="39"/>
+      <c r="R13" s="39"/>
+      <c r="S13" s="39"/>
+      <c r="T13" s="39"/>
+      <c r="U13" s="39"/>
+      <c r="V13" s="39"/>
+      <c r="W13" s="39"/>
+      <c r="X13" s="39" t="s">
+        <v>224</v>
+      </c>
+      <c r="Y13" s="39"/>
+      <c r="Z13" s="39"/>
+      <c r="AA13" s="39"/>
+      <c r="AB13" s="39"/>
+      <c r="AC13" s="39"/>
+      <c r="AD13" s="39"/>
+      <c r="AE13" s="39"/>
+      <c r="AF13" s="39"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AC2" xr:uid="{00000000-0009-0000-0000-000001000000}"/>

</xml_diff>